<commit_message>
feat: add cost estimation documentation and supporting project spreadsheets
</commit_message>
<xml_diff>
--- a/Traffic in Cell Network.xlsx
+++ b/Traffic in Cell Network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\ACS-Cloud\ParabitCloudEnterprise-CostEstimator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E334A97D-5FFF-4207-9F62-0FE43E776C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2115A8C7-32D5-4D93-AF96-75FEC843A26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8534CC66-4B3A-4D6A-9605-08362BAD3903}"/>
   </bookViews>
@@ -764,7 +764,7 @@
     <col min="14" max="14" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.140625" bestFit="1" customWidth="1"/>
@@ -5055,6 +5055,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="45a87b6d-81c1-43eb-a76c-dda31669890c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b66f160e-7eb3-429e-bf83-99c73d74cee8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100129BC0B25D6DF347A98E037D7CED8806" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4aa21137cd32dec5114a2e8197494b58">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b66f160e-7eb3-429e-bf83-99c73d74cee8" xmlns:ns3="45a87b6d-81c1-43eb-a76c-dda31669890c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94b99523bed6575d59999512cb8c9f98" ns2:_="" ns3:_="">
     <xsd:import namespace="b66f160e-7eb3-429e-bf83-99c73d74cee8"/>
@@ -5255,27 +5275,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8E12DC0-087E-4052-BC19-7C1A777396B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e410088d-183d-4878-8fba-05a7d0f012e5"/>
+    <ds:schemaRef ds:uri="c99c58dc-4bca-4617-921a-4bfddcd97dca"/>
+    <ds:schemaRef ds:uri="45a87b6d-81c1-43eb-a76c-dda31669890c"/>
+    <ds:schemaRef ds:uri="b66f160e-7eb3-429e-bf83-99c73d74cee8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="45a87b6d-81c1-43eb-a76c-dda31669890c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b66f160e-7eb3-429e-bf83-99c73d74cee8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17471E1A-DB6D-4D61-ABF2-104C5A9C3ADA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{749F2537-EBBD-495C-A784-F43DD4A790F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5292,31 +5319,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17471E1A-DB6D-4D61-ABF2-104C5A9C3ADA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8E12DC0-087E-4052-BC19-7C1A777396B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e410088d-183d-4878-8fba-05a7d0f012e5"/>
-    <ds:schemaRef ds:uri="c99c58dc-4bca-4617-921a-4bfddcd97dca"/>
-    <ds:schemaRef ds:uri="45a87b6d-81c1-43eb-a76c-dda31669890c"/>
-    <ds:schemaRef ds:uri="b66f160e-7eb3-429e-bf83-99c73d74cee8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>